<commit_message>
all templates with dynamic data
</commit_message>
<xml_diff>
--- a/public/template/ClaimLeadDetailsTemplate.xlsx
+++ b/public/template/ClaimLeadDetailsTemplate.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="MBAUsQgiLBzJFHkCsBMt+Nviy7QmqPas+scTkPL/kIs="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="bfOEjV0OlHYa/bA/KmblNbhg8p892H8tsLWIr9uHjO4="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>Lead ID</t>
   </si>
@@ -33,9 +33,18 @@
     <t>Product</t>
   </si>
   <si>
+    <t>MP NO</t>
+  </si>
+  <si>
     <t>Policy Number</t>
   </si>
   <si>
+    <t>POLICY COVERED</t>
+  </si>
+  <si>
+    <t>Policy Expired Date</t>
+  </si>
+  <si>
     <t>Customer ID</t>
   </si>
   <si>
@@ -45,46 +54,61 @@
     <t>DECEASED NAME</t>
   </si>
   <si>
-    <t>MP NO</t>
-  </si>
-  <si>
-    <t>POLICY COVERED</t>
+    <t>Date of Birth</t>
+  </si>
+  <si>
+    <t>DATE OF DEATH</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>AGE</t>
+  </si>
+  <si>
+    <t>DECEASED</t>
+  </si>
+  <si>
+    <t>DEATH INTIMATION DATE</t>
+  </si>
+  <si>
+    <t>PLACE OF DEATH</t>
+  </si>
+  <si>
+    <t>CAUSE OF DEATH</t>
+  </si>
+  <si>
+    <t>Loan Account ID</t>
   </si>
   <si>
     <t>Loan Tenure</t>
   </si>
   <si>
-    <t>Policy Expired Date</t>
-  </si>
-  <si>
-    <t>DATE OF DEATH</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>DECEASED</t>
-  </si>
-  <si>
-    <t>DEATH INTIMATION DATE</t>
-  </si>
-  <si>
-    <t>AGE</t>
-  </si>
-  <si>
-    <t>PLACE OF DEATH</t>
-  </si>
-  <si>
-    <t>CAUSE OF DEATH</t>
-  </si>
-  <si>
-    <t>Loan Account ID</t>
-  </si>
-  <si>
     <t>CLAIM AMT</t>
   </si>
   <si>
-    <t>Date of Birth</t>
+    <t>Nominee Name</t>
+  </si>
+  <si>
+    <t>RELATIONSHIP</t>
+  </si>
+  <si>
+    <t>Date of document received</t>
+  </si>
+  <si>
+    <t>Processed by</t>
+  </si>
+  <si>
+    <t>Date of submision to partner</t>
+  </si>
+  <si>
+    <t>Date of re-submision to partner</t>
+  </si>
+  <si>
+    <t>HO Remarks</t>
+  </si>
+  <si>
+    <t>Remarks</t>
   </si>
   <si>
     <t>Claim Status</t>
@@ -93,13 +117,67 @@
     <t>CAS Status</t>
   </si>
   <si>
-    <t>Nominee Name</t>
-  </si>
-  <si>
-    <t>RELATIONSHIP</t>
-  </si>
-  <si>
-    <t>Nominee Contact No</t>
+    <t>SPDC/RL Status</t>
+  </si>
+  <si>
+    <t>Notificatiion No</t>
+  </si>
+  <si>
+    <t>Loan Amount</t>
+  </si>
+  <si>
+    <t>Loan Outstanding Amt</t>
+  </si>
+  <si>
+    <t>Payable to Nominee</t>
+  </si>
+  <si>
+    <t>Date of settlement</t>
+  </si>
+  <si>
+    <t>NEFT Rejection Date</t>
+  </si>
+  <si>
+    <t>NEFT Reason For Rejection</t>
+  </si>
+  <si>
+    <t>Final Settlement Date</t>
+  </si>
+  <si>
+    <t>UTRN of MPH</t>
+  </si>
+  <si>
+    <t>UTRN of Nominee</t>
+  </si>
+  <si>
+    <t>Recovery Status</t>
+  </si>
+  <si>
+    <t>Bounced SPDC No</t>
+  </si>
+  <si>
+    <t>SPDC Doposit Date</t>
+  </si>
+  <si>
+    <t>SPDC Bounced Date</t>
+  </si>
+  <si>
+    <t>SPDC Bounced reason</t>
+  </si>
+  <si>
+    <t>Recovered Amount</t>
+  </si>
+  <si>
+    <t>Write off received</t>
+  </si>
+  <si>
+    <t>Write off status</t>
+  </si>
+  <si>
+    <t>Handed over to Business Head</t>
+  </si>
+  <si>
+    <t>Handed over to credit</t>
   </si>
   <si>
     <t>Nominee Name as per Bank Records</t>
@@ -117,12 +195,6 @@
     <t>Bank Branch Name</t>
   </si>
   <si>
-    <t>Loan Outstanding Amt</t>
-  </si>
-  <si>
-    <t>Payable to Nominee</t>
-  </si>
-  <si>
     <t>SPDC-Bank Name</t>
   </si>
   <si>
@@ -135,86 +207,32 @@
     <t>POD Number</t>
   </si>
   <si>
-    <t>CHEQUE SENT DATE</t>
-  </si>
-  <si>
-    <t>ACKNOWLEDGEMENT RECEIVED DATE</t>
+    <t>Nominee Contact Number</t>
+  </si>
+  <si>
+    <t>Branch Remarks</t>
+  </si>
+  <si>
+    <t>Maker at Branch</t>
+  </si>
+  <si>
+    <t>Checker at Branch</t>
+  </si>
+  <si>
+    <t>Ack Received Date</t>
+  </si>
+  <si>
+    <t>SPDC Received Date</t>
   </si>
   <si>
     <t>Packet Number</t>
-  </si>
-  <si>
-    <t>SPDC/RL Status</t>
-  </si>
-  <si>
-    <t>Processed by</t>
-  </si>
-  <si>
-    <t>HO Remarks</t>
-  </si>
-  <si>
-    <t>Date of document received</t>
-  </si>
-  <si>
-    <t>Date of submision to partner</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Date of re-submision to partner</t>
-  </si>
-  <si>
-    <t>Date of settlement</t>
-  </si>
-  <si>
-    <t>NEFT Rejection Date</t>
-  </si>
-  <si>
-    <t>NEFT Reason For Rejection</t>
-  </si>
-  <si>
-    <t>Final Settlement Date</t>
-  </si>
-  <si>
-    <t>Recovery Status</t>
-  </si>
-  <si>
-    <t>Bounced CHQ No</t>
-  </si>
-  <si>
-    <t>CHQ Bounced Date</t>
-  </si>
-  <si>
-    <t>CHQ Bounced reason</t>
-  </si>
-  <si>
-    <t>Write off received</t>
-  </si>
-  <si>
-    <t>Write off status</t>
-  </si>
-  <si>
-    <t>Handed over to Business Head</t>
-  </si>
-  <si>
-    <t>Handed over to credit</t>
-  </si>
-  <si>
-    <t>Branch Remarks</t>
-  </si>
-  <si>
-    <t>Maker at Branch</t>
-  </si>
-  <si>
-    <t>Checker at Branch</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -226,8 +244,25 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
+      <color rgb="FF212529"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFEFEFEF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFEFEFEF"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -242,14 +277,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF999999"/>
-        <bgColor rgb="FF999999"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCCCCC"/>
-        <bgColor rgb="FFCCCCCC"/>
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -259,21 +288,27 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -488,143 +523,143 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="6" width="12.63"/>
+    <col customWidth="1" min="1" max="1" width="21.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AG1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
       <c r="AI1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="4" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="4" t="s">
+      <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="4" t="s">
+      <c r="AL1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="4" t="s">
+      <c r="AM1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="4" t="s">
+      <c r="AN1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AQ1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AR1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AS1" s="1" t="s">
         <v>44</v>
       </c>
       <c r="AT1" s="2" t="s">
@@ -642,37 +677,37 @@
       <c r="AX1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" s="2" t="s">
+      <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" s="2" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" s="2" t="s">
+      <c r="BA1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" s="2" t="s">
+      <c r="BB1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" s="2" t="s">
+      <c r="BC1" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" s="2" t="s">
+      <c r="BD1" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" s="2" t="s">
+      <c r="BE1" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="BF1" s="2" t="s">
+      <c r="BF1" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="BG1" s="2" t="s">
+      <c r="BG1" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" s="2" t="s">
+      <c r="BH1" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" s="2" t="s">
+      <c r="BI1" s="4" t="s">
         <v>60</v>
       </c>
       <c r="BJ1" s="4" t="s">
@@ -681,8 +716,26 @@
       <c r="BK1" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="BL1" s="4" t="s">
+      <c r="BL1" s="5" t="s">
         <v>63</v>
+      </c>
+      <c r="BM1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP1" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ1" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR1" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1"/>
@@ -1641,47 +1694,6 @@
     <row r="955" ht="15.75" customHeight="1"/>
     <row r="956" ht="15.75" customHeight="1"/>
     <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>